<commit_message>
StageLayer LayerName 영어 enum으로(SKY·FAR·MID·PLAY·FRONT·BACK)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDH3mwZmVtgx1ALhFj2DHN
</commit_message>
<xml_diff>
--- a/tables/StageLayer.xlsx
+++ b/tables/StageLayer.xlsx
@@ -460,7 +460,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>한 행 = 스테이지의 배경 레이어 하나. StageID는 Stage ID. Parallax는 카메라 이동 대비 만분율(0=고정, 10000=플레이 레이어와 같이).</t>
+          <t>한 행 = 스테이지의 배경 레이어 하나. StageID는 Stage ID. Parallax는 카메라 이동 대비 만분율(0=고정, 10000=플레이 레이어와 같이). LayerName enum: SKY(하늘), FAR(원경), MID(중경), PLAY(플레이), FRONT(전경), BACK(배경), ImageKey 끝과 같음(10/29 영어로 변경).</t>
         </is>
       </c>
       <c r="C1" s="1" t="n"/>
@@ -606,7 +606,7 @@
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>하늘</t>
+          <t>SKY</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -643,7 +643,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>원경</t>
+          <t>FAR</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -680,7 +680,7 @@
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>중경</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>플레이</t>
+          <t>PLAY</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -754,7 +754,7 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>전경</t>
+          <t>FRONT</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -791,7 +791,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>하늘</t>
+          <t>SKY</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -823,7 +823,7 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>원경</t>
+          <t>FAR</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -855,7 +855,7 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>중경</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -887,7 +887,7 @@
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>플레이</t>
+          <t>PLAY</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -919,7 +919,7 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>하늘</t>
+          <t>SKY</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -951,7 +951,7 @@
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>원경</t>
+          <t>FAR</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -983,7 +983,7 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>중경</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1015,7 +1015,7 @@
       </c>
       <c r="E19" s="3" t="inlineStr">
         <is>
-          <t>플레이</t>
+          <t>PLAY</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -1047,7 +1047,7 @@
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>배경</t>
+          <t>BACK</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>플레이</t>
+          <t>PLAY</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">

</xml_diff>